<commit_message>
Update roster: Export New Roster OCTOBER 2026 Version 3.xlsx
</commit_message>
<xml_diff>
--- a/rosters/.versions/2026-10/current.xlsx
+++ b/rosters/.versions/2026-10/current.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\80235\OneDrive - Oman Air\Desktop\Rosters\STAFF OPERATION SCHEDULE\Roster 5 x 3\2026\OPS\10 October 2026\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{40008CBF-61AE-48EB-9D54-B1BB89EB89BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{EE87734E-B5A9-4CF5-9F13-95385DBC9D23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="2" activeTab="2" xr2:uid="{9736B67C-D61B-41E1-B07B-429B3D8AE9CC}"/>
   </bookViews>
@@ -60,7 +60,7 @@
     <author>Rodolfo C Magcaling</author>
   </authors>
   <commentList>
-    <comment ref="I5" authorId="0" shapeId="0" xr:uid="{E5B95F7E-7FE7-4ACA-8105-3771BA8AEFAC}">
+    <comment ref="I5" authorId="0" shapeId="0" xr:uid="{1FB28473-83AC-48A2-A25E-A048AD3569B5}">
       <text>
         <r>
           <rPr>
@@ -84,7 +84,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J6" authorId="0" shapeId="0" xr:uid="{C76FBE1B-49BF-44BE-98A6-6A88BCF213BF}">
+    <comment ref="J6" authorId="0" shapeId="0" xr:uid="{0D642D8A-0622-478C-AA8C-26138A21D067}">
       <text>
         <r>
           <rPr>
@@ -108,7 +108,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="I7" authorId="0" shapeId="0" xr:uid="{EE90E9F6-FADB-4B65-9658-182404D53C6A}">
+    <comment ref="I7" authorId="0" shapeId="0" xr:uid="{5B8D31DC-1978-43D5-851A-74B929C76278}">
       <text>
         <r>
           <rPr>
@@ -132,7 +132,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J7" authorId="0" shapeId="0" xr:uid="{626C6050-1C54-4CDD-BC3D-8DE96D9B9350}">
+    <comment ref="J7" authorId="0" shapeId="0" xr:uid="{5D9C2106-0605-46FB-9B70-32714C1F0A3B}">
       <text>
         <r>
           <rPr>
@@ -156,7 +156,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="M7" authorId="0" shapeId="0" xr:uid="{41EFAABE-0D91-4B7A-AD01-625808329262}">
+    <comment ref="M7" authorId="0" shapeId="0" xr:uid="{29A2C595-8BB3-476B-AC86-BE2F510163C4}">
       <text>
         <r>
           <rPr>
@@ -180,7 +180,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="W7" authorId="0" shapeId="0" xr:uid="{4F02542B-1375-466B-A28D-EAF15E38E4BA}">
+    <comment ref="W7" authorId="0" shapeId="0" xr:uid="{3130FC4A-4921-40ED-B1AC-EF7A819F140C}">
       <text>
         <r>
           <rPr>
@@ -204,7 +204,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="X7" authorId="0" shapeId="0" xr:uid="{5A9D05C2-B47D-4738-A9A1-20CADBEA6A31}">
+    <comment ref="X7" authorId="0" shapeId="0" xr:uid="{DC009075-5C75-4A7A-AD1C-DC9B02CACAB3}">
       <text>
         <r>
           <rPr>
@@ -228,7 +228,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AD7" authorId="0" shapeId="0" xr:uid="{2E2B34CD-59E9-4DDA-84A4-D778D7011FD5}">
+    <comment ref="AD7" authorId="0" shapeId="0" xr:uid="{E5DDB41D-8779-4077-9246-8115C9DEF48C}">
       <text>
         <r>
           <rPr>
@@ -252,7 +252,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="K8" authorId="0" shapeId="0" xr:uid="{44B63640-5BC8-4F7F-9692-32D1BA16875C}">
+    <comment ref="K8" authorId="0" shapeId="0" xr:uid="{B8E4DBA2-ACF5-4663-BCCF-6031BF5BBDE7}">
       <text>
         <r>
           <rPr>
@@ -276,7 +276,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Y8" authorId="0" shapeId="0" xr:uid="{E91E56F6-37BF-4ECC-916C-CC51C3D6F426}">
+    <comment ref="Y8" authorId="0" shapeId="0" xr:uid="{530699A9-0A13-480D-848E-D8FC58CE7329}">
       <text>
         <r>
           <rPr>
@@ -300,7 +300,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="I9" authorId="0" shapeId="0" xr:uid="{75A7E804-CE42-47DF-91BA-56842D688ABE}">
+    <comment ref="I9" authorId="0" shapeId="0" xr:uid="{84CBB52C-F61F-4D5C-86E2-593BA5229401}">
       <text>
         <r>
           <rPr>
@@ -324,7 +324,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="P9" authorId="0" shapeId="0" xr:uid="{38EC3420-AB56-4267-A1B8-4FFA1F8C884D}">
+    <comment ref="P9" authorId="0" shapeId="0" xr:uid="{9E0C0A75-4DA1-45A8-AE64-FF115422110A}">
       <text>
         <r>
           <rPr>
@@ -348,7 +348,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AH13" authorId="0" shapeId="0" xr:uid="{89904727-D895-4B94-A30B-E8A850D0B7AD}">
+    <comment ref="AH13" authorId="0" shapeId="0" xr:uid="{A5C5D7C8-F494-40D6-9E08-721AB2B7472A}">
       <text>
         <r>
           <rPr>
@@ -372,7 +372,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J14" authorId="0" shapeId="0" xr:uid="{056A3FAB-8F7F-470D-B7E5-D4B02D1C1C1E}">
+    <comment ref="J14" authorId="0" shapeId="0" xr:uid="{575C54EE-BD0B-45C2-BAC2-5BA9FF09213E}">
       <text>
         <r>
           <rPr>
@@ -396,7 +396,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="I15" authorId="0" shapeId="0" xr:uid="{C7DEA02F-FFFB-4B91-880F-D320A6EDD8A5}">
+    <comment ref="I15" authorId="0" shapeId="0" xr:uid="{937B14A7-64C0-4DCC-A90E-BEA18C74A651}">
       <text>
         <r>
           <rPr>
@@ -420,7 +420,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="O15" authorId="0" shapeId="0" xr:uid="{84360FE1-84C8-48C5-91B5-37393F324F62}">
+    <comment ref="O15" authorId="0" shapeId="0" xr:uid="{800B12B5-4288-4608-9266-7416B396A3EB}">
       <text>
         <r>
           <rPr>
@@ -444,7 +444,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="P15" authorId="0" shapeId="0" xr:uid="{E612757E-32BA-4D8B-9725-027033107ABB}">
+    <comment ref="P15" authorId="0" shapeId="0" xr:uid="{9E294EB2-635D-43A0-8E8B-27DB10752DB2}">
       <text>
         <r>
           <rPr>
@@ -468,7 +468,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Q15" authorId="0" shapeId="0" xr:uid="{DB24E70C-C870-4CF2-A121-13A6CA089124}">
+    <comment ref="Q15" authorId="0" shapeId="0" xr:uid="{1655273A-2102-4B41-9A84-C888C6AC4E6D}">
       <text>
         <r>
           <rPr>
@@ -492,7 +492,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AD15" authorId="0" shapeId="0" xr:uid="{2853906F-23D2-4893-BDF8-15B652FAC93E}">
+    <comment ref="AD15" authorId="0" shapeId="0" xr:uid="{2CDAF01C-3F91-4AC7-865D-34CB334F0BD6}">
       <text>
         <r>
           <rPr>
@@ -516,7 +516,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AE15" authorId="0" shapeId="0" xr:uid="{361AC406-19E9-4611-A134-8DD7931BB638}">
+    <comment ref="AE15" authorId="0" shapeId="0" xr:uid="{ED616A99-EC43-4D15-BB5E-6B1665D9FDC8}">
       <text>
         <r>
           <rPr>
@@ -540,7 +540,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AF15" authorId="0" shapeId="0" xr:uid="{57698312-09A2-4AB6-AA7E-82ED436AA765}">
+    <comment ref="AF15" authorId="0" shapeId="0" xr:uid="{EE2D1A3E-85EA-46D8-B83F-C3921C34D4FD}">
       <text>
         <r>
           <rPr>
@@ -564,7 +564,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AG15" authorId="0" shapeId="0" xr:uid="{20C7CB2F-6038-4E4A-A86A-2ED95412F670}">
+    <comment ref="AG15" authorId="0" shapeId="0" xr:uid="{C2458652-20F6-4853-9ADD-605E1FC8B97C}">
       <text>
         <r>
           <rPr>
@@ -588,7 +588,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AH15" authorId="0" shapeId="0" xr:uid="{0DDC0084-0558-4450-B845-2DC9ECEE5117}">
+    <comment ref="AH15" authorId="0" shapeId="0" xr:uid="{8E8CDA36-692E-4292-B131-ED306D9C3B77}">
       <text>
         <r>
           <rPr>
@@ -612,7 +612,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="K20" authorId="0" shapeId="0" xr:uid="{D44F74D3-76D7-4DD5-9133-F8987472AE02}">
+    <comment ref="K20" authorId="0" shapeId="0" xr:uid="{4B4D59D3-14A5-45D6-A267-EFDDB7709A61}">
       <text>
         <r>
           <rPr>
@@ -636,7 +636,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="P20" authorId="0" shapeId="0" xr:uid="{74EC443E-B71E-4F27-BE50-17BB54BACB2C}">
+    <comment ref="P20" authorId="0" shapeId="0" xr:uid="{05E2A9D8-387C-4E0B-8F74-174BD4E1D38D}">
       <text>
         <r>
           <rPr>
@@ -660,7 +660,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Q20" authorId="0" shapeId="0" xr:uid="{88E572D0-0630-4CC7-AED6-3270D3C7CB1F}">
+    <comment ref="Q20" authorId="0" shapeId="0" xr:uid="{37766D7C-0DF8-4459-B117-3039EB518999}">
       <text>
         <r>
           <rPr>
@@ -684,7 +684,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="I21" authorId="0" shapeId="0" xr:uid="{647F29C4-421E-4838-86C6-50CA94E9D344}">
+    <comment ref="I21" authorId="0" shapeId="0" xr:uid="{49BED592-2D84-421E-A3D9-46F5F45FE501}">
       <text>
         <r>
           <rPr>
@@ -708,7 +708,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="P22" authorId="0" shapeId="0" xr:uid="{484FC985-157F-40EF-984F-0CF56AC3A63E}">
+    <comment ref="P22" authorId="0" shapeId="0" xr:uid="{5580DE47-442D-43E3-AC72-7A5F00217F18}">
       <text>
         <r>
           <rPr>
@@ -732,7 +732,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="M23" authorId="0" shapeId="0" xr:uid="{CBC37A8E-57B2-4F30-BC1E-A96B6B0227A6}">
+    <comment ref="M23" authorId="0" shapeId="0" xr:uid="{A469C8AC-3BBD-490A-B9B8-490D5600D15E}">
       <text>
         <r>
           <rPr>
@@ -756,7 +756,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AG23" authorId="0" shapeId="0" xr:uid="{4CB0431C-F6DF-4F83-AB44-DD4EB279B51A}">
+    <comment ref="AG23" authorId="0" shapeId="0" xr:uid="{A744EC60-B16D-4E5D-895F-397B9333F093}">
       <text>
         <r>
           <rPr>
@@ -780,7 +780,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="T24" authorId="0" shapeId="0" xr:uid="{5CCC2C69-2425-415E-A5FA-1B8354FDAF77}">
+    <comment ref="T24" authorId="0" shapeId="0" xr:uid="{65AB467B-BD21-4524-80CC-AC98721DC81C}">
       <text>
         <r>
           <rPr>
@@ -804,7 +804,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="L25" authorId="0" shapeId="0" xr:uid="{370550EA-ADF1-4935-B023-5B2673BC021D}">
+    <comment ref="L25" authorId="0" shapeId="0" xr:uid="{0A9CD046-3B9B-4C6A-B597-1734D3072487}">
       <text>
         <r>
           <rPr>
@@ -828,7 +828,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="T26" authorId="0" shapeId="0" xr:uid="{65EB856C-66D9-4718-9A51-EA6E805E3080}">
+    <comment ref="T26" authorId="0" shapeId="0" xr:uid="{A512605E-6755-474C-AC67-C9DEA87443D1}">
       <text>
         <r>
           <rPr>
@@ -852,7 +852,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J28" authorId="0" shapeId="0" xr:uid="{07316C2C-7B44-420B-B548-2E29612E18AB}">
+    <comment ref="J28" authorId="0" shapeId="0" xr:uid="{4B5007DE-6D81-47AF-9747-3C25BEE94DB2}">
       <text>
         <r>
           <rPr>
@@ -876,7 +876,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="R28" authorId="0" shapeId="0" xr:uid="{CBEAE7AF-EF06-4369-8EE3-A2EE7DC488C0}">
+    <comment ref="R28" authorId="0" shapeId="0" xr:uid="{BE4472CC-C5DA-4736-B1DD-88A7864E302D}">
       <text>
         <r>
           <rPr>
@@ -900,7 +900,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="S28" authorId="0" shapeId="0" xr:uid="{7A874946-268D-4591-84AE-8B7E69C85A3F}">
+    <comment ref="S28" authorId="0" shapeId="0" xr:uid="{99897B9B-20A0-48BE-97C8-0DD576046EA0}">
       <text>
         <r>
           <rPr>
@@ -924,7 +924,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AH28" authorId="0" shapeId="0" xr:uid="{9B33E08C-C233-40AD-AEAE-9353B401B8E8}">
+    <comment ref="AH28" authorId="0" shapeId="0" xr:uid="{132C8BC0-ACDD-4273-8F0E-94A2DA2102AB}">
       <text>
         <r>
           <rPr>
@@ -948,7 +948,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="P30" authorId="0" shapeId="0" xr:uid="{4DC1D242-CE13-48DC-B40E-3AC77BFA48C7}">
+    <comment ref="P30" authorId="0" shapeId="0" xr:uid="{580913E6-520B-40CC-BCE0-2EDC88626641}">
       <text>
         <r>
           <rPr>
@@ -972,7 +972,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="M32" authorId="0" shapeId="0" xr:uid="{3B1332DF-95CC-4863-B51D-5625BF08C8C3}">
+    <comment ref="M32" authorId="0" shapeId="0" xr:uid="{586E0B95-E8FF-4A4D-A602-CDE396BE55E1}">
       <text>
         <r>
           <rPr>
@@ -996,7 +996,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="L35" authorId="0" shapeId="0" xr:uid="{406A13A2-60A9-404B-8356-577C93222FAF}">
+    <comment ref="L35" authorId="0" shapeId="0" xr:uid="{3BAACA3D-0D03-49C4-AD10-2220943078DC}">
       <text>
         <r>
           <rPr>
@@ -1020,7 +1020,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="K38" authorId="0" shapeId="0" xr:uid="{F5413401-D99A-4264-AB93-D96D53809A6F}">
+    <comment ref="K38" authorId="0" shapeId="0" xr:uid="{9D1FE4D1-E439-4D70-AC82-F90716B35905}">
       <text>
         <r>
           <rPr>
@@ -1044,7 +1044,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="M41" authorId="0" shapeId="0" xr:uid="{14421B94-B268-4240-8EA0-77BA9E6A3EC4}">
+    <comment ref="M41" authorId="0" shapeId="0" xr:uid="{4BAF1E7A-84E7-4F62-A070-4649FA58B06B}">
       <text>
         <r>
           <rPr>
@@ -1068,7 +1068,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="P41" authorId="0" shapeId="0" xr:uid="{715D1387-E90F-4527-A1A2-E18C1B6C809D}">
+    <comment ref="P41" authorId="0" shapeId="0" xr:uid="{17DC3F4C-EC7A-4F52-AFEF-8FE24F4EDB88}">
       <text>
         <r>
           <rPr>
@@ -1092,7 +1092,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AG42" authorId="0" shapeId="0" xr:uid="{B12D28E6-2AB5-4211-A1A9-6C9BF6D0BD69}">
+    <comment ref="AG42" authorId="0" shapeId="0" xr:uid="{4D701E8F-AF03-48B5-9A55-07AACCC0D32E}">
       <text>
         <r>
           <rPr>
@@ -1116,7 +1116,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="T43" authorId="0" shapeId="0" xr:uid="{D78C45C7-51B1-48D7-A14E-B86D53EA7CCE}">
+    <comment ref="T43" authorId="0" shapeId="0" xr:uid="{0F479FEF-DACC-43D5-AC76-96BD6459DBB8}">
       <text>
         <r>
           <rPr>
@@ -1140,7 +1140,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="X47" authorId="0" shapeId="0" xr:uid="{F947DF51-2292-411A-B44F-1E6505E4F896}">
+    <comment ref="X47" authorId="0" shapeId="0" xr:uid="{91A3640B-3268-4E40-B6CD-5903DCEC98B5}">
       <text>
         <r>
           <rPr>
@@ -1164,7 +1164,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AE49" authorId="0" shapeId="0" xr:uid="{21C9BABE-6AB3-4E97-B6B1-3CF18D0A28CB}">
+    <comment ref="AE49" authorId="0" shapeId="0" xr:uid="{EE148A49-EDC4-4ECF-B360-BC43A0A61D40}">
       <text>
         <r>
           <rPr>
@@ -1188,7 +1188,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="T51" authorId="0" shapeId="0" xr:uid="{399AA536-F6B8-4156-9C16-04E48A6CCA29}">
+    <comment ref="T51" authorId="0" shapeId="0" xr:uid="{3B8ADE25-70FA-4C89-8BE9-B06FECFE90F0}">
       <text>
         <r>
           <rPr>
@@ -1212,7 +1212,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AA51" authorId="0" shapeId="0" xr:uid="{27C9FA1A-D397-49B7-AB6C-622E77ACC420}">
+    <comment ref="AA51" authorId="0" shapeId="0" xr:uid="{E3779567-82A2-4321-96CD-DCED25C76D65}">
       <text>
         <r>
           <rPr>
@@ -1236,7 +1236,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AG51" authorId="0" shapeId="0" xr:uid="{0EF371DB-DA66-478C-98BA-09C3D94EFAF5}">
+    <comment ref="AG51" authorId="0" shapeId="0" xr:uid="{406FC0E1-72FE-4E8B-A094-F17785E01D95}">
       <text>
         <r>
           <rPr>
@@ -1260,7 +1260,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AA56" authorId="0" shapeId="0" xr:uid="{5D054998-DBC6-4FD5-B587-FB9B62A9DD98}">
+    <comment ref="AA56" authorId="0" shapeId="0" xr:uid="{3877DDEB-2D6E-4916-8E28-A2E12B91E95E}">
       <text>
         <r>
           <rPr>
@@ -1284,7 +1284,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AH56" authorId="0" shapeId="0" xr:uid="{78E4F77A-28AB-4B9E-A6F0-DEE122D525F7}">
+    <comment ref="AH56" authorId="0" shapeId="0" xr:uid="{AE24A25E-E2A4-4A8D-9C02-F0F9F4E3E58E}">
       <text>
         <r>
           <rPr>
@@ -1308,7 +1308,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="L57" authorId="0" shapeId="0" xr:uid="{1205396F-7D8E-46A4-9A2D-D5D84C51F268}">
+    <comment ref="L57" authorId="0" shapeId="0" xr:uid="{F21347E5-25D3-4ED1-B8F4-9D39073B745C}">
       <text>
         <r>
           <rPr>
@@ -1332,7 +1332,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="K59" authorId="0" shapeId="0" xr:uid="{5F1116E2-5ED4-477A-A53F-32DE835FD13E}">
+    <comment ref="K59" authorId="0" shapeId="0" xr:uid="{8CC2DE01-76BF-4973-B8C4-1D02BA6CCD67}">
       <text>
         <r>
           <rPr>
@@ -1356,7 +1356,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="AH59" authorId="0" shapeId="0" xr:uid="{449349D3-EE15-479F-A7E5-7E3475E65328}">
+    <comment ref="AH59" authorId="0" shapeId="0" xr:uid="{D532CE5B-20A9-453E-BD0A-8016CD46219D}">
       <text>
         <r>
           <rPr>
@@ -1380,7 +1380,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="M60" authorId="0" shapeId="0" xr:uid="{B6E51678-F58F-4EC5-BD36-ABB7926E4EB4}">
+    <comment ref="M60" authorId="0" shapeId="0" xr:uid="{0700576D-B558-412F-BB27-143C7D348A29}">
       <text>
         <r>
           <rPr>
@@ -1404,7 +1404,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="L63" authorId="0" shapeId="0" xr:uid="{DE335AB0-FD60-4A1F-B9ED-9B8389E834A2}">
+    <comment ref="L63" authorId="0" shapeId="0" xr:uid="{DCE16F0E-4B2F-4BC7-8A25-8FC1C481B112}">
       <text>
         <r>
           <rPr>
@@ -1428,7 +1428,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="S64" authorId="0" shapeId="0" xr:uid="{3546162E-8DE2-4590-A9AB-EAE25A00001E}">
+    <comment ref="S64" authorId="0" shapeId="0" xr:uid="{FEE8C6CB-83B7-4A68-A1E5-452D902CB7D0}">
       <text>
         <r>
           <rPr>
@@ -1452,7 +1452,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="M65" authorId="0" shapeId="0" xr:uid="{D693CB87-1C45-4839-A2FC-7AA291A33368}">
+    <comment ref="M65" authorId="0" shapeId="0" xr:uid="{8B728466-C03D-42AB-B275-DEA9EAB4F488}">
       <text>
         <r>
           <rPr>
@@ -1476,7 +1476,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="I68" authorId="0" shapeId="0" xr:uid="{66C697F9-137F-4F58-902C-90AB817B0F83}">
+    <comment ref="I68" authorId="0" shapeId="0" xr:uid="{B135192E-4998-4DEA-8B6D-B40023EEAF03}">
       <text>
         <r>
           <rPr>
@@ -1500,7 +1500,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="M70" authorId="0" shapeId="0" xr:uid="{DABE30CE-43BD-4C52-A81A-445BFC31152B}">
+    <comment ref="M70" authorId="0" shapeId="0" xr:uid="{EF3E1E24-6BE8-46DB-883B-1884DD1A24AE}">
       <text>
         <r>
           <rPr>
@@ -1524,7 +1524,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="X74" authorId="0" shapeId="0" xr:uid="{35953405-B476-47E8-A0D8-74E2329218AC}">
+    <comment ref="X74" authorId="0" shapeId="0" xr:uid="{177E5F48-EC67-4D90-B9BD-DC051FE1352F}">
       <text>
         <r>
           <rPr>
@@ -5144,7 +5144,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="266">
+  <cellXfs count="269">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="15" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -5907,11 +5907,1623 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="340">
+  <dxfs count="528">
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <fgColor auto="1"/>
+          <bgColor theme="5" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.14996795556505021"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF7030A0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B0F0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.14996795556505021"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF7030A0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC00000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC00000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC00000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B0F0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.14996795556505021"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC00000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC00000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF7030A0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC00000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC00000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B0F0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.14996795556505021"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF7030A0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC00000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC00000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC00000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FFFF0000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B0F0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.14996795556505021"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.14996795556505021"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF7030A0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC00000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC00000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC00000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FFFF0000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B0F0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.14996795556505021"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF7030A0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC00000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC00000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC00000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FFFF0000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B0F0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.14996795556505021"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.14996795556505021"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF7030A0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC00000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC00000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC00000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FFFF0000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B0F0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.14996795556505021"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC00000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC00000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF7030A0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC00000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC00000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B0F0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.14996795556505021"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC00000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC00000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF7030A0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC00000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC00000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B0F0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.14996795556505021"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF7030A0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC00000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC00000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC00000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B0F0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.14996795556505021"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC00000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC00000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF7030A0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC00000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC00000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B0F0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.14996795556505021"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF7030A0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC00000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC00000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC00000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FFFF0000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B0F0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.14996795556505021"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.14996795556505021"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF7030A0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC00000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC00000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC00000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <color rgb="FFFF0000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFFFF00"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FF00B0F0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <color auto="1"/>
@@ -14835,26 +16447,26 @@
     <mergeCell ref="AC2:AF2"/>
   </mergeCells>
   <conditionalFormatting sqref="E8:AI37 AK8:AN37 E39:AI42">
-    <cfRule type="expression" dxfId="339" priority="4">
+    <cfRule type="expression" dxfId="527" priority="4">
       <formula>LEFT(E8,1)="N"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="338" priority="5">
+    <cfRule type="expression" dxfId="526" priority="5">
       <formula>LEFT(E8,1)="A"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="337" priority="7">
+    <cfRule type="expression" dxfId="525" priority="7">
       <formula>LEFT(E8,1)="M"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="336" priority="8">
+    <cfRule type="expression" dxfId="524" priority="8">
       <formula>LEFT(E8,1)="D"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E39:AI42 E8:AI37 AK8:AN37">
-    <cfRule type="expression" dxfId="335" priority="3">
+    <cfRule type="expression" dxfId="523" priority="3">
       <formula>LEFT(E8,1)="O"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E39:AI42">
-    <cfRule type="expression" dxfId="334" priority="1">
+    <cfRule type="expression" dxfId="522" priority="1">
       <formula>ISEVEN(ROW($E39))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -15549,19 +17161,19 @@
         <v>219</v>
       </c>
       <c r="R8" s="128" t="s">
-        <v>194</v>
+        <v>253</v>
       </c>
       <c r="S8" s="128" t="s">
-        <v>194</v>
+        <v>253</v>
       </c>
       <c r="T8" s="128" t="s">
-        <v>195</v>
+        <v>253</v>
       </c>
       <c r="U8" s="128" t="s">
-        <v>195</v>
+        <v>253</v>
       </c>
       <c r="V8" s="128" t="s">
-        <v>195</v>
+        <v>253</v>
       </c>
       <c r="W8" s="128" t="s">
         <v>219</v>
@@ -15611,11 +17223,11 @@
       </c>
       <c r="AM8" s="93">
         <f t="shared" si="1"/>
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="AN8" s="93">
         <f t="shared" si="2"/>
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="AO8" s="93">
         <f t="shared" si="3"/>
@@ -16168,28 +17780,28 @@
         <v>253</v>
       </c>
       <c r="U13" s="49" t="s">
-        <v>219</v>
+        <v>253</v>
       </c>
       <c r="V13" s="49" t="s">
-        <v>219</v>
+        <v>253</v>
       </c>
       <c r="W13" s="49" t="s">
-        <v>194</v>
+        <v>253</v>
       </c>
       <c r="X13" s="49" t="s">
-        <v>194</v>
+        <v>253</v>
       </c>
       <c r="Y13" s="49" t="s">
-        <v>195</v>
+        <v>253</v>
       </c>
       <c r="Z13" s="49" t="s">
-        <v>218</v>
+        <v>253</v>
       </c>
       <c r="AA13" s="49" t="s">
-        <v>218</v>
+        <v>253</v>
       </c>
       <c r="AB13" s="49" t="s">
-        <v>219</v>
+        <v>253</v>
       </c>
       <c r="AC13" s="49" t="s">
         <v>219</v>
@@ -16222,19 +17834,19 @@
       </c>
       <c r="AM13" s="48">
         <f t="shared" si="6"/>
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="AN13" s="48">
         <f t="shared" si="7"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AO13" s="48">
         <f t="shared" si="8"/>
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AP13" s="48">
         <f t="shared" si="9"/>
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="14" spans="2:42" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
@@ -16552,7 +18164,7 @@
         <v>218</v>
       </c>
       <c r="Z16" s="96" t="s">
-        <v>239</v>
+        <v>219</v>
       </c>
       <c r="AA16" s="96" t="s">
         <v>219</v>
@@ -17269,7 +18881,7 @@
         <v>218</v>
       </c>
       <c r="S22" s="96" t="s">
-        <v>219</v>
+        <v>239</v>
       </c>
       <c r="T22" s="96" t="s">
         <v>219</v>
@@ -17413,7 +19025,7 @@
         <v>218</v>
       </c>
       <c r="Z23" s="96" t="s">
-        <v>219</v>
+        <v>239</v>
       </c>
       <c r="AA23" s="96" t="s">
         <v>219</v>
@@ -18019,22 +19631,22 @@
         <v>219</v>
       </c>
       <c r="W28" s="106" t="s">
-        <v>253</v>
+        <v>194</v>
       </c>
       <c r="X28" s="106" t="s">
-        <v>253</v>
+        <v>194</v>
       </c>
       <c r="Y28" s="106" t="s">
-        <v>253</v>
+        <v>195</v>
       </c>
       <c r="Z28" s="106" t="s">
-        <v>253</v>
+        <v>218</v>
       </c>
       <c r="AA28" s="125" t="s">
-        <v>253</v>
+        <v>218</v>
       </c>
       <c r="AB28" s="106" t="s">
-        <v>253</v>
+        <v>219</v>
       </c>
       <c r="AC28" s="106" t="s">
         <v>219</v>
@@ -18066,19 +19678,19 @@
       </c>
       <c r="AM28" s="48">
         <f t="shared" si="11"/>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="AN28" s="48">
         <f t="shared" si="12"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AO28" s="48">
         <f t="shared" si="13"/>
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="AP28" s="48">
         <f t="shared" si="14"/>
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="29" spans="2:42" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
@@ -18889,19 +20501,19 @@
         <v>194</v>
       </c>
       <c r="AB35" s="96" t="s">
-        <v>194</v>
+        <v>253</v>
       </c>
       <c r="AC35" s="96" t="s">
-        <v>195</v>
+        <v>253</v>
       </c>
       <c r="AD35" s="96" t="s">
-        <v>218</v>
+        <v>253</v>
       </c>
       <c r="AE35" s="96" t="s">
-        <v>218</v>
+        <v>253</v>
       </c>
       <c r="AF35" s="96" t="s">
-        <v>219</v>
+        <v>253</v>
       </c>
       <c r="AG35" s="96" t="s">
         <v>219</v>
@@ -18921,19 +20533,19 @@
       </c>
       <c r="AM35" s="48">
         <f t="shared" si="16"/>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AN35" s="48">
         <f t="shared" si="17"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AO35" s="48">
         <f t="shared" si="18"/>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="AP35" s="48">
         <f t="shared" si="19"/>
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="36" spans="2:42" ht="18.75" x14ac:dyDescent="0.25">
@@ -19432,52 +21044,52 @@
         <v>139</v>
       </c>
       <c r="D40" s="146"/>
-      <c r="F40" s="96" t="s">
+      <c r="F40" s="268" t="s">
         <v>255</v>
       </c>
-      <c r="G40" s="96" t="s">
+      <c r="G40" s="268" t="s">
         <v>255</v>
       </c>
-      <c r="H40" s="96" t="s">
+      <c r="H40" s="268" t="s">
         <v>255</v>
       </c>
-      <c r="I40" s="96" t="s">
+      <c r="I40" s="268" t="s">
         <v>255</v>
       </c>
-      <c r="J40" s="96" t="s">
+      <c r="J40" s="268" t="s">
         <v>255</v>
       </c>
-      <c r="K40" s="96" t="s">
+      <c r="K40" s="268" t="s">
         <v>255</v>
       </c>
-      <c r="L40" s="96" t="s">
+      <c r="L40" s="268" t="s">
         <v>255</v>
       </c>
-      <c r="M40" s="96" t="s">
+      <c r="M40" s="268" t="s">
         <v>255</v>
       </c>
-      <c r="N40" s="96" t="s">
+      <c r="N40" s="268" t="s">
         <v>255</v>
       </c>
-      <c r="O40" s="96" t="s">
+      <c r="O40" s="268" t="s">
         <v>255</v>
       </c>
-      <c r="P40" s="96" t="s">
+      <c r="P40" s="268" t="s">
         <v>255</v>
       </c>
-      <c r="Q40" s="96" t="s">
+      <c r="Q40" s="268" t="s">
         <v>255</v>
       </c>
-      <c r="R40" s="96" t="s">
+      <c r="R40" s="268" t="s">
         <v>255</v>
       </c>
-      <c r="S40" s="96" t="s">
+      <c r="S40" s="268" t="s">
         <v>255</v>
       </c>
-      <c r="T40" s="96" t="s">
+      <c r="T40" s="268" t="s">
         <v>255</v>
       </c>
-      <c r="U40" s="96" t="s">
+      <c r="U40" s="268" t="s">
         <v>255</v>
       </c>
       <c r="V40" s="96" t="s">
@@ -19746,10 +21358,10 @@
         <v>194</v>
       </c>
       <c r="AC42" s="96" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="AD42" s="96" t="s">
-        <v>195</v>
+        <v>218</v>
       </c>
       <c r="AE42" s="96" t="s">
         <v>218</v>
@@ -19775,7 +21387,7 @@
       </c>
       <c r="AM42" s="48">
         <f t="shared" si="16"/>
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="AN42" s="48">
         <f t="shared" si="17"/>
@@ -19783,7 +21395,7 @@
       </c>
       <c r="AO42" s="48">
         <f t="shared" si="18"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AP42" s="48">
         <f t="shared" si="19"/>
@@ -20329,7 +21941,7 @@
         <v>219</v>
       </c>
       <c r="T47" s="96" t="s">
-        <v>219</v>
+        <v>239</v>
       </c>
       <c r="U47" s="96" t="s">
         <v>219</v>
@@ -20481,7 +22093,7 @@
         <v>194</v>
       </c>
       <c r="AD48" s="96" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="AE48" s="96" t="s">
         <v>195</v>
@@ -20507,11 +22119,11 @@
       </c>
       <c r="AM48" s="48">
         <f t="shared" si="16"/>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AN48" s="48">
         <f t="shared" si="17"/>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AO48" s="48">
         <f t="shared" si="18"/>
@@ -22284,7 +23896,7 @@
         <v>195</v>
       </c>
       <c r="AE63" s="96" t="s">
-        <v>195</v>
+        <v>253</v>
       </c>
       <c r="AF63" s="96" t="s">
         <v>218</v>
@@ -22311,7 +23923,7 @@
       </c>
       <c r="AN63" s="48">
         <f t="shared" si="17"/>
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="AO63" s="48">
         <f t="shared" si="18"/>
@@ -22739,7 +24351,7 @@
         <v>218</v>
       </c>
       <c r="T67" s="94" t="s">
-        <v>219</v>
+        <v>239</v>
       </c>
       <c r="U67" s="94" t="s">
         <v>219</v>
@@ -22977,7 +24589,7 @@
         <v>242</v>
       </c>
       <c r="R69" s="95" t="s">
-        <v>219</v>
+        <v>240</v>
       </c>
       <c r="S69" s="96" t="s">
         <v>194</v>
@@ -23102,7 +24714,7 @@
         <v>219</v>
       </c>
       <c r="S70" s="94" t="s">
-        <v>219</v>
+        <v>242</v>
       </c>
       <c r="T70" s="94" t="s">
         <v>194</v>
@@ -23217,20 +24829,20 @@
       <c r="P71" s="96" t="s">
         <v>219</v>
       </c>
-      <c r="Q71" s="94" t="s">
-        <v>194</v>
-      </c>
-      <c r="R71" s="94" t="s">
-        <v>194</v>
-      </c>
-      <c r="S71" s="94" t="s">
-        <v>195</v>
-      </c>
-      <c r="T71" s="94" t="s">
-        <v>218</v>
-      </c>
-      <c r="U71" s="95" t="s">
-        <v>218</v>
+      <c r="Q71" s="266" t="s">
+        <v>255</v>
+      </c>
+      <c r="R71" s="266" t="s">
+        <v>255</v>
+      </c>
+      <c r="S71" s="266" t="s">
+        <v>255</v>
+      </c>
+      <c r="T71" s="266" t="s">
+        <v>255</v>
+      </c>
+      <c r="U71" s="267" t="s">
+        <v>255</v>
       </c>
       <c r="V71" s="96" t="s">
         <v>219</v>
@@ -23283,15 +24895,15 @@
       </c>
       <c r="AM71" s="48">
         <f t="shared" si="16"/>
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AN71" s="48">
         <f t="shared" si="17"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AO71" s="48">
         <f t="shared" si="18"/>
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AP71" s="48">
         <f t="shared" si="19"/>
@@ -23645,7 +25257,7 @@
       </c>
       <c r="AN75" s="48">
         <f t="shared" ref="AN75:AN86" si="22">COUNTIF($F63:$AJ63,"A*")</f>
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="AO75" s="48">
         <f t="shared" ref="AO75:AO86" si="23">COUNTIF($F63:$AJ63,"N*")</f>
@@ -23708,11 +25320,11 @@
       </c>
       <c r="Q76" s="37">
         <f t="shared" si="25"/>
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="R76" s="37">
         <f t="shared" si="25"/>
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="S76" s="37">
         <f t="shared" si="25"/>
@@ -23752,15 +25364,15 @@
       </c>
       <c r="AB76" s="37">
         <f t="shared" si="25"/>
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="AC76" s="37">
         <f t="shared" si="25"/>
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="AD76" s="37">
         <f t="shared" si="25"/>
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="AE76" s="37">
         <f t="shared" si="25"/>
@@ -23867,7 +25479,7 @@
       </c>
       <c r="S77" s="37">
         <f t="shared" si="26"/>
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="T77" s="37">
         <f t="shared" si="26"/>
@@ -23915,7 +25527,7 @@
       </c>
       <c r="AE77" s="37">
         <f t="shared" si="26"/>
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="AF77" s="37">
         <f t="shared" si="26"/>
@@ -24022,11 +25634,11 @@
       </c>
       <c r="T78" s="37">
         <f t="shared" si="27"/>
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="U78" s="37">
         <f t="shared" si="27"/>
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="V78" s="37">
         <f t="shared" si="27"/>
@@ -24066,7 +25678,7 @@
       </c>
       <c r="AE78" s="37">
         <f t="shared" si="27"/>
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="AF78" s="37">
         <f t="shared" si="27"/>
@@ -24221,7 +25833,7 @@
       </c>
       <c r="AF79" s="37">
         <f t="shared" si="28"/>
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="AG79" s="37">
         <f t="shared" si="28"/>
@@ -24618,15 +26230,15 @@
       </c>
       <c r="R82" s="51">
         <f t="shared" si="31"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S82" s="51">
         <f t="shared" si="31"/>
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="T82" s="51">
         <f t="shared" si="31"/>
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="U82" s="51">
         <f t="shared" si="31"/>
@@ -24754,15 +26366,15 @@
       </c>
       <c r="AM83" s="48">
         <f t="shared" si="21"/>
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AN83" s="48">
         <f t="shared" si="22"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AO83" s="48">
         <f t="shared" si="23"/>
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AP83" s="48">
         <f t="shared" si="24"/>
@@ -24821,23 +26433,23 @@
       </c>
       <c r="Q84" s="41">
         <f t="shared" si="32"/>
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="R84" s="41">
         <f t="shared" si="32"/>
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="S84" s="41">
         <f t="shared" si="32"/>
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="T84" s="41">
         <f t="shared" si="32"/>
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="U84" s="41">
         <f t="shared" si="32"/>
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="V84" s="41">
         <f t="shared" si="32"/>
@@ -24865,19 +26477,19 @@
       </c>
       <c r="AB84" s="41">
         <f t="shared" si="32"/>
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="AC84" s="41">
         <f t="shared" si="32"/>
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="AD84" s="41">
         <f t="shared" si="32"/>
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="AE84" s="41">
         <f t="shared" si="32"/>
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="AF84" s="41">
         <f t="shared" si="32"/>
@@ -25091,23 +26703,23 @@
       </c>
       <c r="Q86" s="37">
         <f t="shared" si="33"/>
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="R86" s="37">
         <f t="shared" si="33"/>
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="S86" s="37">
         <f t="shared" si="33"/>
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="T86" s="37">
         <f t="shared" si="33"/>
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="U86" s="37">
         <f t="shared" si="33"/>
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="V86" s="37">
         <f t="shared" si="33"/>
@@ -25135,23 +26747,23 @@
       </c>
       <c r="AB86" s="37">
         <f t="shared" si="33"/>
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="AC86" s="37">
         <f t="shared" si="33"/>
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="AD86" s="37">
         <f t="shared" si="33"/>
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AE86" s="37">
         <f t="shared" si="33"/>
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="AF86" s="37">
         <f t="shared" si="33"/>
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="AG86" s="37">
         <f t="shared" si="33"/>
@@ -26410,19 +28022,19 @@
         <v>219</v>
       </c>
       <c r="R8" s="128" t="s">
-        <v>194</v>
+        <v>253</v>
       </c>
       <c r="S8" s="128" t="s">
-        <v>194</v>
+        <v>253</v>
       </c>
       <c r="T8" s="128" t="s">
-        <v>195</v>
+        <v>253</v>
       </c>
       <c r="U8" s="128" t="s">
-        <v>195</v>
+        <v>253</v>
       </c>
       <c r="V8" s="128" t="s">
-        <v>195</v>
+        <v>253</v>
       </c>
       <c r="W8" s="128" t="s">
         <v>219</v>
@@ -26472,11 +28084,11 @@
       </c>
       <c r="AM8" s="48">
         <f t="shared" si="1"/>
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="AN8" s="48">
         <f t="shared" si="2"/>
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="AO8" s="48">
         <f t="shared" si="3"/>
@@ -26577,11 +28189,11 @@
       </c>
       <c r="R10" s="37">
         <f t="shared" si="5"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S10" s="37">
         <f t="shared" si="5"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="T10" s="37">
         <f t="shared" si="5"/>
@@ -26716,15 +28328,15 @@
       </c>
       <c r="T11" s="37">
         <f t="shared" si="6"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U11" s="37">
         <f t="shared" si="6"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V11" s="37">
         <f t="shared" si="6"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="W11" s="37">
         <f t="shared" si="6"/>
@@ -27363,23 +28975,23 @@
       </c>
       <c r="R16" s="51">
         <f t="shared" si="11"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S16" s="51">
         <f t="shared" si="11"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T16" s="51">
         <f t="shared" si="11"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U16" s="51">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="V16" s="51">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="W16" s="51">
         <f t="shared" si="11"/>
@@ -27530,23 +29142,23 @@
       </c>
       <c r="R18" s="41">
         <f t="shared" si="12"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="S18" s="41">
         <f t="shared" si="12"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="T18" s="41">
         <f t="shared" si="12"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="U18" s="41">
         <f t="shared" si="12"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="V18" s="41">
         <f t="shared" si="12"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="W18" s="41">
         <f t="shared" si="12"/>
@@ -27760,23 +29372,23 @@
       </c>
       <c r="R20" s="37">
         <f t="shared" si="13"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="S20" s="37">
         <f t="shared" si="13"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="T20" s="37">
         <f t="shared" si="13"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="U20" s="37">
         <f t="shared" si="13"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="V20" s="37">
         <f t="shared" si="13"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="W20" s="37">
         <f t="shared" si="13"/>
@@ -27953,28 +29565,28 @@
   </mergeCells>
   <phoneticPr fontId="14" type="noConversion"/>
   <conditionalFormatting sqref="F5:AJ8">
-    <cfRule type="containsText" dxfId="270" priority="1" operator="containsText" text="AN13">
+    <cfRule type="containsText" dxfId="458" priority="1" operator="containsText" text="AN13">
       <formula>NOT(ISERROR(SEARCH("AN13",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="269" priority="2" operator="containsText" text="MN06">
+    <cfRule type="containsText" dxfId="457" priority="2" operator="containsText" text="MN06">
       <formula>NOT(ISERROR(SEARCH("MN06",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="268" priority="3" operator="containsText" text="LV">
+    <cfRule type="containsText" dxfId="456" priority="3" operator="containsText" text="LV">
       <formula>NOT(ISERROR(SEARCH("LV",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="267" priority="4" operator="containsText" text="AN13">
+    <cfRule type="containsText" dxfId="455" priority="4" operator="containsText" text="AN13">
       <formula>NOT(ISERROR(SEARCH("AN13",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="266" priority="5" operator="containsText" text="MN06">
+    <cfRule type="containsText" dxfId="454" priority="5" operator="containsText" text="MN06">
       <formula>NOT(ISERROR(SEARCH("MN06",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="265" priority="7" operator="containsText" text="TR">
+    <cfRule type="containsText" dxfId="453" priority="7" operator="containsText" text="TR">
       <formula>NOT(ISERROR(SEARCH("TR",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="264" priority="10" operator="containsText" text="OFF">
+    <cfRule type="containsText" dxfId="452" priority="10" operator="containsText" text="OFF">
       <formula>NOT(ISERROR(SEARCH("OFF",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="263" priority="11" operator="containsText" text="ME07">
+    <cfRule type="containsText" dxfId="451" priority="11" operator="containsText" text="ME07">
       <formula>NOT(ISERROR(SEARCH("ME07",F5)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -28801,28 +30413,28 @@
         <v>253</v>
       </c>
       <c r="U9" s="49" t="s">
-        <v>219</v>
+        <v>253</v>
       </c>
       <c r="V9" s="49" t="s">
-        <v>219</v>
+        <v>253</v>
       </c>
       <c r="W9" s="49" t="s">
-        <v>194</v>
+        <v>253</v>
       </c>
       <c r="X9" s="49" t="s">
-        <v>194</v>
+        <v>253</v>
       </c>
       <c r="Y9" s="49" t="s">
-        <v>195</v>
+        <v>253</v>
       </c>
       <c r="Z9" s="49" t="s">
-        <v>218</v>
+        <v>253</v>
       </c>
       <c r="AA9" s="49" t="s">
-        <v>218</v>
+        <v>253</v>
       </c>
       <c r="AB9" s="49" t="s">
-        <v>219</v>
+        <v>253</v>
       </c>
       <c r="AC9" s="49" t="s">
         <v>219</v>
@@ -28855,19 +30467,19 @@
       </c>
       <c r="AM9" s="48">
         <f t="shared" si="1"/>
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="AN9" s="48">
         <f t="shared" si="2"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AO9" s="48">
         <f t="shared" si="3"/>
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AP9" s="48">
         <f t="shared" si="4"/>
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10" spans="2:42" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
@@ -29102,11 +30714,11 @@
       </c>
       <c r="W12" s="37">
         <f t="shared" si="5"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="X12" s="37">
         <f t="shared" si="5"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Y12" s="37">
         <f t="shared" si="5"/>
@@ -29241,7 +30853,7 @@
       </c>
       <c r="Y13" s="37">
         <f t="shared" si="6"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Z13" s="37">
         <f t="shared" si="6"/>
@@ -29376,11 +30988,11 @@
       </c>
       <c r="Z14" s="37">
         <f t="shared" si="7"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AA14" s="37">
         <f t="shared" si="7"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AB14" s="37">
         <f t="shared" si="7"/>
@@ -29487,11 +31099,11 @@
       </c>
       <c r="U15" s="37">
         <f t="shared" si="8"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="V15" s="37">
         <f t="shared" si="8"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="W15" s="37">
         <f t="shared" si="8"/>
@@ -29515,7 +31127,7 @@
       </c>
       <c r="AB15" s="37">
         <f t="shared" si="8"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AC15" s="37">
         <f t="shared" si="8"/>
@@ -30055,23 +31667,23 @@
       </c>
       <c r="W20" s="41">
         <f t="shared" si="12"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="X20" s="41">
         <f t="shared" si="12"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Y20" s="41">
         <f t="shared" si="12"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="Z20" s="41">
         <f t="shared" si="12"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AA20" s="41">
         <f t="shared" si="12"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AB20" s="41">
         <f t="shared" si="12"/>
@@ -30277,35 +31889,35 @@
       </c>
       <c r="U22" s="37">
         <f t="shared" si="13"/>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="V22" s="37">
         <f t="shared" si="13"/>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="W22" s="37">
         <f t="shared" si="13"/>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="X22" s="37">
         <f t="shared" si="13"/>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="Y22" s="37">
         <f t="shared" si="13"/>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="Z22" s="37">
         <f t="shared" si="13"/>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AA22" s="37">
         <f t="shared" si="13"/>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AB22" s="37">
         <f t="shared" si="13"/>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AC22" s="37">
         <f t="shared" si="13"/>
@@ -30560,46 +32172,46 @@
   </mergeCells>
   <phoneticPr fontId="14" type="noConversion"/>
   <conditionalFormatting sqref="F5:AJ10">
-    <cfRule type="containsText" dxfId="262" priority="1" operator="containsText" text="NN21">
+    <cfRule type="containsText" dxfId="450" priority="1" operator="containsText" text="NN21">
       <formula>NOT(ISERROR(SEARCH("NN21",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="261" priority="2" operator="containsText" text="AN13">
+    <cfRule type="containsText" dxfId="449" priority="2" operator="containsText" text="AN13">
       <formula>NOT(ISERROR(SEARCH("AN13",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="260" priority="3" operator="containsText" text="MN06">
+    <cfRule type="containsText" dxfId="448" priority="3" operator="containsText" text="MN06">
       <formula>NOT(ISERROR(SEARCH("MN06",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="259" priority="4" operator="containsText" text="OT">
+    <cfRule type="containsText" dxfId="447" priority="4" operator="containsText" text="OT">
       <formula>NOT(ISERROR(SEARCH("OT",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="258" priority="5" operator="containsText" text="NN21">
+    <cfRule type="containsText" dxfId="446" priority="5" operator="containsText" text="NN21">
       <formula>NOT(ISERROR(SEARCH("NN21",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="257" priority="6" operator="containsText" text="MN06">
+    <cfRule type="containsText" dxfId="445" priority="6" operator="containsText" text="MN06">
       <formula>NOT(ISERROR(SEARCH("MN06",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="256" priority="7" operator="containsText" text="AN13">
+    <cfRule type="containsText" dxfId="444" priority="7" operator="containsText" text="AN13">
       <formula>NOT(ISERROR(SEARCH("AN13",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="255" priority="8" operator="containsText" text="LV">
+    <cfRule type="containsText" dxfId="443" priority="8" operator="containsText" text="LV">
       <formula>NOT(ISERROR(SEARCH("LV",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="254" priority="9" operator="containsText" text="STNN21">
+    <cfRule type="containsText" dxfId="442" priority="9" operator="containsText" text="STNN21">
       <formula>NOT(ISERROR(SEARCH("STNN21",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="253" priority="10" operator="containsText" text="STAN13">
+    <cfRule type="containsText" dxfId="441" priority="10" operator="containsText" text="STAN13">
       <formula>NOT(ISERROR(SEARCH("STAN13",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="252" priority="11" operator="containsText" text="STMN06">
+    <cfRule type="containsText" dxfId="440" priority="11" operator="containsText" text="STMN06">
       <formula>NOT(ISERROR(SEARCH("STMN06",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="251" priority="12" operator="containsText" text="MN12">
+    <cfRule type="containsText" dxfId="439" priority="12" operator="containsText" text="MN12">
       <formula>NOT(ISERROR(SEARCH("MN12",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="250" priority="13" operator="containsText" text="TR">
+    <cfRule type="containsText" dxfId="438" priority="13" operator="containsText" text="TR">
       <formula>NOT(ISERROR(SEARCH("TR",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="249" priority="14" operator="containsText" text="OFF">
+    <cfRule type="containsText" dxfId="437" priority="14" operator="containsText" text="OFF">
       <formula>NOT(ISERROR(SEARCH("OFF",F5)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -31073,7 +32685,7 @@
         <v>218</v>
       </c>
       <c r="Z6" s="96" t="s">
-        <v>239</v>
+        <v>219</v>
       </c>
       <c r="AA6" s="96" t="s">
         <v>219</v>
@@ -31784,7 +33396,7 @@
         <v>218</v>
       </c>
       <c r="S12" s="96" t="s">
-        <v>219</v>
+        <v>239</v>
       </c>
       <c r="T12" s="96" t="s">
         <v>219</v>
@@ -31927,7 +33539,7 @@
         <v>218</v>
       </c>
       <c r="Z13" s="96" t="s">
-        <v>219</v>
+        <v>239</v>
       </c>
       <c r="AA13" s="96" t="s">
         <v>219</v>
@@ -32528,22 +34140,22 @@
         <v>219</v>
       </c>
       <c r="W18" s="106" t="s">
-        <v>253</v>
+        <v>194</v>
       </c>
       <c r="X18" s="106" t="s">
-        <v>253</v>
+        <v>194</v>
       </c>
       <c r="Y18" s="106" t="s">
-        <v>253</v>
+        <v>195</v>
       </c>
       <c r="Z18" s="106" t="s">
-        <v>253</v>
+        <v>218</v>
       </c>
       <c r="AA18" s="125" t="s">
-        <v>253</v>
+        <v>218</v>
       </c>
       <c r="AB18" s="106" t="s">
-        <v>253</v>
+        <v>219</v>
       </c>
       <c r="AC18" s="106" t="s">
         <v>219</v>
@@ -32575,19 +34187,19 @@
       </c>
       <c r="AM18" s="48">
         <f t="shared" si="1"/>
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="AN18" s="48">
         <f t="shared" si="2"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AO18" s="48">
         <f t="shared" si="3"/>
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="AP18" s="48">
         <f t="shared" si="4"/>
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="19" spans="2:42" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
@@ -32823,11 +34435,11 @@
       </c>
       <c r="W21" s="37">
         <f t="shared" si="5"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="X21" s="37">
         <f t="shared" si="5"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Y21" s="37">
         <f t="shared" si="5"/>
@@ -32962,7 +34574,7 @@
       </c>
       <c r="Y22" s="37">
         <f t="shared" si="6"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Z22" s="37">
         <f t="shared" si="6"/>
@@ -33097,11 +34709,11 @@
       </c>
       <c r="Z23" s="37">
         <f t="shared" si="7"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AA23" s="37">
         <f t="shared" si="7"/>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="AB23" s="37">
         <f t="shared" si="7"/>
@@ -33236,7 +34848,7 @@
       </c>
       <c r="AB24" s="37">
         <f t="shared" si="8"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AC24" s="37">
         <f t="shared" si="8"/>
@@ -33462,7 +35074,7 @@
       </c>
       <c r="S26" s="51">
         <f t="shared" si="10"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T26" s="51">
         <f t="shared" si="10"/>
@@ -33645,23 +35257,23 @@
       </c>
       <c r="W28" s="41">
         <f t="shared" si="11"/>
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="X28" s="41">
         <f t="shared" si="11"/>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="Y28" s="41">
         <f t="shared" si="11"/>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="Z28" s="41">
         <f t="shared" si="11"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AA28" s="41">
         <f t="shared" si="11"/>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AB28" s="41">
         <f t="shared" si="11"/>
@@ -33875,27 +35487,27 @@
       </c>
       <c r="W30" s="37">
         <f t="shared" si="12"/>
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="X30" s="37">
         <f t="shared" si="12"/>
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="Y30" s="37">
         <f t="shared" si="12"/>
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="Z30" s="37">
         <f t="shared" si="12"/>
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="AA30" s="37">
         <f t="shared" si="12"/>
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="AB30" s="37">
         <f t="shared" si="12"/>
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="AC30" s="37">
         <f t="shared" si="12"/>
@@ -34158,46 +35770,46 @@
   </mergeCells>
   <phoneticPr fontId="14" type="noConversion"/>
   <conditionalFormatting sqref="F5:AJ19">
-    <cfRule type="containsText" dxfId="248" priority="1" operator="containsText" text="AN13">
+    <cfRule type="containsText" dxfId="436" priority="1" operator="containsText" text="AN13">
       <formula>NOT(ISERROR(SEARCH("AN13",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="247" priority="2" operator="containsText" text="NN21">
+    <cfRule type="containsText" dxfId="435" priority="2" operator="containsText" text="NN21">
       <formula>NOT(ISERROR(SEARCH("NN21",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="246" priority="3" operator="containsText" text="MN06">
+    <cfRule type="containsText" dxfId="434" priority="3" operator="containsText" text="MN06">
       <formula>NOT(ISERROR(SEARCH("MN06",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="245" priority="5" operator="containsText" text="OT">
+    <cfRule type="containsText" dxfId="433" priority="5" operator="containsText" text="OT">
       <formula>NOT(ISERROR(SEARCH("OT",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="244" priority="6" operator="containsText" text="NN21">
+    <cfRule type="containsText" dxfId="432" priority="6" operator="containsText" text="NN21">
       <formula>NOT(ISERROR(SEARCH("NN21",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="243" priority="7" operator="containsText" text="AN13">
+    <cfRule type="containsText" dxfId="431" priority="7" operator="containsText" text="AN13">
       <formula>NOT(ISERROR(SEARCH("AN13",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="242" priority="8" operator="containsText" text="MN06">
+    <cfRule type="containsText" dxfId="430" priority="8" operator="containsText" text="MN06">
       <formula>NOT(ISERROR(SEARCH("MN06",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="241" priority="9" operator="containsText" text="STMN06">
+    <cfRule type="containsText" dxfId="429" priority="9" operator="containsText" text="STMN06">
       <formula>NOT(ISERROR(SEARCH("STMN06",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="240" priority="11" operator="containsText" text="STAN13">
+    <cfRule type="containsText" dxfId="428" priority="11" operator="containsText" text="STAN13">
       <formula>NOT(ISERROR(SEARCH("STAN13",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="239" priority="12" operator="containsText" text="TR">
+    <cfRule type="containsText" dxfId="427" priority="12" operator="containsText" text="TR">
       <formula>NOT(ISERROR(SEARCH("TR",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="238" priority="13" operator="containsText" text="LV">
+    <cfRule type="containsText" dxfId="426" priority="13" operator="containsText" text="LV">
       <formula>NOT(ISERROR(SEARCH("LV",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="237" priority="18" operator="containsText" text="STAN13">
+    <cfRule type="containsText" dxfId="425" priority="18" operator="containsText" text="STAN13">
       <formula>NOT(ISERROR(SEARCH("STAN13",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="236" priority="19" operator="containsText" text="STNN21">
+    <cfRule type="containsText" dxfId="424" priority="19" operator="containsText" text="STNN21">
       <formula>NOT(ISERROR(SEARCH("STNN21",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="235" priority="21" operator="containsText" text="OFF">
+    <cfRule type="containsText" dxfId="423" priority="21" operator="containsText" text="OFF">
       <formula>NOT(ISERROR(SEARCH("OFF",F5)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -35168,19 +36780,19 @@
         <v>194</v>
       </c>
       <c r="AB10" s="96" t="s">
-        <v>194</v>
+        <v>253</v>
       </c>
       <c r="AC10" s="96" t="s">
-        <v>195</v>
+        <v>253</v>
       </c>
       <c r="AD10" s="96" t="s">
-        <v>218</v>
+        <v>253</v>
       </c>
       <c r="AE10" s="96" t="s">
-        <v>218</v>
+        <v>253</v>
       </c>
       <c r="AF10" s="96" t="s">
-        <v>219</v>
+        <v>253</v>
       </c>
       <c r="AG10" s="96" t="s">
         <v>219</v>
@@ -35200,19 +36812,19 @@
       </c>
       <c r="AM10" s="48">
         <f t="shared" si="1"/>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AN10" s="48">
         <f t="shared" si="2"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AO10" s="48">
         <f t="shared" si="3"/>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="AP10" s="48">
         <f t="shared" si="4"/>
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="11" spans="2:42" ht="18.75" x14ac:dyDescent="0.25">
@@ -35711,52 +37323,52 @@
         <v>139</v>
       </c>
       <c r="D15" s="146"/>
-      <c r="F15" s="96" t="s">
+      <c r="F15" s="268" t="s">
         <v>255</v>
       </c>
-      <c r="G15" s="96" t="s">
+      <c r="G15" s="268" t="s">
         <v>255</v>
       </c>
-      <c r="H15" s="96" t="s">
+      <c r="H15" s="268" t="s">
         <v>255</v>
       </c>
-      <c r="I15" s="96" t="s">
+      <c r="I15" s="268" t="s">
         <v>255</v>
       </c>
-      <c r="J15" s="96" t="s">
+      <c r="J15" s="268" t="s">
         <v>255</v>
       </c>
-      <c r="K15" s="96" t="s">
+      <c r="K15" s="268" t="s">
         <v>255</v>
       </c>
-      <c r="L15" s="96" t="s">
+      <c r="L15" s="268" t="s">
         <v>255</v>
       </c>
-      <c r="M15" s="96" t="s">
+      <c r="M15" s="268" t="s">
         <v>255</v>
       </c>
-      <c r="N15" s="96" t="s">
+      <c r="N15" s="268" t="s">
         <v>255</v>
       </c>
-      <c r="O15" s="96" t="s">
+      <c r="O15" s="268" t="s">
         <v>255</v>
       </c>
-      <c r="P15" s="96" t="s">
+      <c r="P15" s="268" t="s">
         <v>255</v>
       </c>
-      <c r="Q15" s="96" t="s">
+      <c r="Q15" s="268" t="s">
         <v>255</v>
       </c>
-      <c r="R15" s="96" t="s">
+      <c r="R15" s="268" t="s">
         <v>255</v>
       </c>
-      <c r="S15" s="96" t="s">
+      <c r="S15" s="268" t="s">
         <v>255</v>
       </c>
-      <c r="T15" s="96" t="s">
+      <c r="T15" s="268" t="s">
         <v>255</v>
       </c>
-      <c r="U15" s="96" t="s">
+      <c r="U15" s="268" t="s">
         <v>255</v>
       </c>
       <c r="V15" s="96" t="s">
@@ -36025,10 +37637,10 @@
         <v>194</v>
       </c>
       <c r="AC17" s="96" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="AD17" s="96" t="s">
-        <v>195</v>
+        <v>218</v>
       </c>
       <c r="AE17" s="96" t="s">
         <v>218</v>
@@ -36054,7 +37666,7 @@
       </c>
       <c r="AM17" s="48">
         <f t="shared" si="1"/>
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="AN17" s="48">
         <f t="shared" si="2"/>
@@ -36062,7 +37674,7 @@
       </c>
       <c r="AO17" s="48">
         <f t="shared" si="3"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AP17" s="48">
         <f t="shared" si="4"/>
@@ -36608,7 +38220,7 @@
         <v>219</v>
       </c>
       <c r="T22" s="96" t="s">
-        <v>219</v>
+        <v>239</v>
       </c>
       <c r="U22" s="96" t="s">
         <v>219</v>
@@ -36760,7 +38372,7 @@
         <v>194</v>
       </c>
       <c r="AD23" s="96" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="AE23" s="96" t="s">
         <v>195</v>
@@ -36786,11 +38398,11 @@
       </c>
       <c r="AM23" s="48">
         <f t="shared" si="1"/>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AN23" s="48">
         <f t="shared" si="2"/>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AO23" s="48">
         <f t="shared" si="3"/>
@@ -38395,15 +40007,15 @@
       </c>
       <c r="AB37" s="37">
         <f t="shared" si="5"/>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AC37" s="37">
         <f t="shared" si="5"/>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AD37" s="37">
         <f t="shared" si="5"/>
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="AE37" s="37">
         <f t="shared" si="5"/>
@@ -38669,7 +40281,7 @@
       </c>
       <c r="AE39" s="37">
         <f t="shared" si="7"/>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AF39" s="37">
         <f t="shared" si="7"/>
@@ -38804,7 +40416,7 @@
       </c>
       <c r="AF40" s="37">
         <f t="shared" si="8"/>
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="AG40" s="37">
         <f t="shared" si="8"/>
@@ -39149,7 +40761,7 @@
       </c>
       <c r="T43" s="51">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U43" s="51">
         <f t="shared" si="11"/>
@@ -39348,19 +40960,19 @@
       </c>
       <c r="AB45" s="41">
         <f t="shared" si="12"/>
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="AC45" s="41">
         <f t="shared" si="12"/>
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="AD45" s="41">
         <f t="shared" si="12"/>
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="AE45" s="41">
         <f t="shared" si="12"/>
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="AF45" s="41">
         <f t="shared" si="12"/>
@@ -39578,23 +41190,23 @@
       </c>
       <c r="AB47" s="37">
         <f t="shared" si="13"/>
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="AC47" s="37">
         <f t="shared" si="13"/>
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="AD47" s="37">
         <f t="shared" si="13"/>
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="AE47" s="37">
         <f t="shared" si="13"/>
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="AF47" s="37">
         <f t="shared" si="13"/>
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="AG47" s="37">
         <f t="shared" si="13"/>
@@ -39858,58 +41470,58 @@
   </mergeCells>
   <phoneticPr fontId="14" type="noConversion"/>
   <conditionalFormatting sqref="F5:AJ35">
-    <cfRule type="containsText" dxfId="234" priority="1" operator="containsText" text="OFF">
+    <cfRule type="containsText" dxfId="422" priority="1" operator="containsText" text="OFF">
       <formula>NOT(ISERROR(SEARCH("OFF",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="233" priority="2" operator="containsText" text="OFF">
+    <cfRule type="containsText" dxfId="421" priority="2" operator="containsText" text="OFF">
       <formula>NOT(ISERROR(SEARCH("OFF",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="232" priority="3" operator="containsText" text="MN06">
+    <cfRule type="containsText" dxfId="420" priority="3" operator="containsText" text="MN06">
       <formula>NOT(ISERROR(SEARCH("MN06",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="231" priority="4" operator="containsText" text="OFF">
+    <cfRule type="containsText" dxfId="419" priority="4" operator="containsText" text="OFF">
       <formula>NOT(ISERROR(SEARCH("OFF",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="230" priority="5" operator="containsText" text="NN21">
+    <cfRule type="containsText" dxfId="418" priority="5" operator="containsText" text="NN21">
       <formula>NOT(ISERROR(SEARCH("NN21",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="229" priority="6" operator="containsText" text="AN13">
+    <cfRule type="containsText" dxfId="417" priority="6" operator="containsText" text="AN13">
       <formula>NOT(ISERROR(SEARCH("AN13",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="228" priority="7" operator="containsText" text="MN06">
+    <cfRule type="containsText" dxfId="416" priority="7" operator="containsText" text="MN06">
       <formula>NOT(ISERROR(SEARCH("MN06",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="227" priority="8" operator="containsText" text="NN21">
+    <cfRule type="containsText" dxfId="415" priority="8" operator="containsText" text="NN21">
       <formula>NOT(ISERROR(SEARCH("NN21",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="226" priority="9" operator="containsText" text="AN13">
+    <cfRule type="containsText" dxfId="414" priority="9" operator="containsText" text="AN13">
       <formula>NOT(ISERROR(SEARCH("AN13",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="225" priority="10" operator="containsText" text="MN06">
+    <cfRule type="containsText" dxfId="413" priority="10" operator="containsText" text="MN06">
       <formula>NOT(ISERROR(SEARCH("MN06",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="224" priority="11" operator="containsText" text="OT">
+    <cfRule type="containsText" dxfId="412" priority="11" operator="containsText" text="OT">
       <formula>NOT(ISERROR(SEARCH("OT",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="223" priority="14" operator="containsText" text="MN12">
+    <cfRule type="containsText" dxfId="411" priority="14" operator="containsText" text="MN12">
       <formula>NOT(ISERROR(SEARCH("MN12",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="222" priority="15" operator="containsText" text="STNN21">
+    <cfRule type="containsText" dxfId="410" priority="15" operator="containsText" text="STNN21">
       <formula>NOT(ISERROR(SEARCH("STNN21",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="221" priority="16" operator="containsText" text="STAN13">
+    <cfRule type="containsText" dxfId="409" priority="16" operator="containsText" text="STAN13">
       <formula>NOT(ISERROR(SEARCH("STAN13",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="220" priority="17" operator="containsText" text="STMN06">
+    <cfRule type="containsText" dxfId="408" priority="17" operator="containsText" text="STMN06">
       <formula>NOT(ISERROR(SEARCH("STMN06",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="219" priority="18" operator="containsText" text="LV">
+    <cfRule type="containsText" dxfId="407" priority="18" operator="containsText" text="LV">
       <formula>NOT(ISERROR(SEARCH("LV",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="218" priority="19" operator="containsText" text="TR">
+    <cfRule type="containsText" dxfId="406" priority="19" operator="containsText" text="TR">
       <formula>NOT(ISERROR(SEARCH("TR",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="217" priority="23" operator="containsText" text="OFF">
+    <cfRule type="containsText" dxfId="405" priority="23" operator="containsText" text="OFF">
       <formula>NOT(ISERROR(SEARCH("OFF",F5)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -40505,7 +42117,7 @@
         <v>195</v>
       </c>
       <c r="AE7" s="96" t="s">
-        <v>195</v>
+        <v>253</v>
       </c>
       <c r="AF7" s="96" t="s">
         <v>218</v>
@@ -40532,7 +42144,7 @@
       </c>
       <c r="AN7" s="22">
         <f t="shared" si="2"/>
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="AO7" s="22">
         <f t="shared" si="3"/>
@@ -40960,7 +42572,7 @@
         <v>218</v>
       </c>
       <c r="T11" s="94" t="s">
-        <v>219</v>
+        <v>239</v>
       </c>
       <c r="U11" s="94" t="s">
         <v>219</v>
@@ -41198,7 +42810,7 @@
         <v>242</v>
       </c>
       <c r="R13" s="95" t="s">
-        <v>219</v>
+        <v>240</v>
       </c>
       <c r="S13" s="96" t="s">
         <v>194</v>
@@ -41323,7 +42935,7 @@
         <v>219</v>
       </c>
       <c r="S14" s="94" t="s">
-        <v>219</v>
+        <v>242</v>
       </c>
       <c r="T14" s="94" t="s">
         <v>194</v>
@@ -41438,20 +43050,20 @@
       <c r="P15" s="96" t="s">
         <v>219</v>
       </c>
-      <c r="Q15" s="94" t="s">
-        <v>194</v>
-      </c>
-      <c r="R15" s="94" t="s">
-        <v>194</v>
-      </c>
-      <c r="S15" s="94" t="s">
-        <v>195</v>
-      </c>
-      <c r="T15" s="94" t="s">
-        <v>218</v>
-      </c>
-      <c r="U15" s="95" t="s">
-        <v>218</v>
+      <c r="Q15" s="266" t="s">
+        <v>255</v>
+      </c>
+      <c r="R15" s="266" t="s">
+        <v>255</v>
+      </c>
+      <c r="S15" s="266" t="s">
+        <v>255</v>
+      </c>
+      <c r="T15" s="266" t="s">
+        <v>255</v>
+      </c>
+      <c r="U15" s="267" t="s">
+        <v>255</v>
       </c>
       <c r="V15" s="96" t="s">
         <v>219</v>
@@ -41504,15 +43116,15 @@
       </c>
       <c r="AM15" s="22">
         <f t="shared" si="1"/>
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AN15" s="22">
         <f t="shared" si="2"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AO15" s="22">
         <f t="shared" si="3"/>
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AP15" s="22">
         <f t="shared" si="4"/>
@@ -41909,11 +43521,11 @@
       </c>
       <c r="Q20" s="37">
         <f t="shared" si="5"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="R20" s="37">
         <f t="shared" si="5"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="S20" s="37">
         <f t="shared" si="5"/>
@@ -42048,7 +43660,7 @@
       </c>
       <c r="S21" s="37">
         <f t="shared" si="6"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="T21" s="37">
         <f t="shared" si="6"/>
@@ -42096,7 +43708,7 @@
       </c>
       <c r="AE21" s="37">
         <f t="shared" si="6"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AF21" s="37">
         <f t="shared" si="6"/>
@@ -42183,11 +43795,11 @@
       </c>
       <c r="T22" s="37">
         <f t="shared" si="7"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U22" s="37">
         <f t="shared" si="7"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="V22" s="37">
         <f t="shared" si="7"/>
@@ -42699,15 +44311,15 @@
       </c>
       <c r="R26" s="51">
         <f t="shared" si="11"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="S26" s="51">
         <f t="shared" si="11"/>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="T26" s="51">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U26" s="51">
         <f t="shared" si="11"/>
@@ -42862,23 +44474,23 @@
       </c>
       <c r="Q28" s="41">
         <f t="shared" si="12"/>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="R28" s="41">
         <f t="shared" si="12"/>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="S28" s="41">
         <f t="shared" si="12"/>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="T28" s="41">
         <f t="shared" si="12"/>
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="U28" s="41">
         <f t="shared" si="12"/>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="V28" s="41">
         <f t="shared" si="12"/>
@@ -42918,7 +44530,7 @@
       </c>
       <c r="AE28" s="41">
         <f t="shared" si="12"/>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="AF28" s="41">
         <f t="shared" si="12"/>
@@ -43093,23 +44705,23 @@
       </c>
       <c r="Q30" s="37">
         <f t="shared" si="13"/>
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="R30" s="37">
         <f t="shared" si="13"/>
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="S30" s="37">
         <f t="shared" si="13"/>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="T30" s="37">
         <f t="shared" si="13"/>
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="U30" s="37">
         <f t="shared" si="13"/>
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="V30" s="37">
         <f t="shared" si="13"/>
@@ -43149,7 +44761,7 @@
       </c>
       <c r="AE30" s="37">
         <f t="shared" si="13"/>
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="AF30" s="37">
         <f t="shared" si="13"/>
@@ -43400,46 +45012,46 @@
   </mergeCells>
   <phoneticPr fontId="14" type="noConversion"/>
   <conditionalFormatting sqref="F5:AJ18">
-    <cfRule type="containsText" dxfId="216" priority="1" operator="containsText" text="AN13">
+    <cfRule type="containsText" dxfId="404" priority="1" operator="containsText" text="AN13">
       <formula>NOT(ISERROR(SEARCH("AN13",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="215" priority="2" operator="containsText" text="NN21">
+    <cfRule type="containsText" dxfId="403" priority="2" operator="containsText" text="NN21">
       <formula>NOT(ISERROR(SEARCH("NN21",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="214" priority="3" operator="containsText" text="MN06">
+    <cfRule type="containsText" dxfId="402" priority="3" operator="containsText" text="MN06">
       <formula>NOT(ISERROR(SEARCH("MN06",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="213" priority="4" operator="containsText" text="OT">
+    <cfRule type="containsText" dxfId="401" priority="4" operator="containsText" text="OT">
       <formula>NOT(ISERROR(SEARCH("OT",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="212" priority="5" operator="containsText" text="MN06">
+    <cfRule type="containsText" dxfId="400" priority="5" operator="containsText" text="MN06">
       <formula>NOT(ISERROR(SEARCH("MN06",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="211" priority="6" operator="containsText" text="NN21">
+    <cfRule type="containsText" dxfId="399" priority="6" operator="containsText" text="NN21">
       <formula>NOT(ISERROR(SEARCH("NN21",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="210" priority="7" operator="containsText" text="AN13">
+    <cfRule type="containsText" dxfId="398" priority="7" operator="containsText" text="AN13">
       <formula>NOT(ISERROR(SEARCH("AN13",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="209" priority="10" operator="containsText" text="STMN06">
+    <cfRule type="containsText" dxfId="397" priority="10" operator="containsText" text="STMN06">
       <formula>NOT(ISERROR(SEARCH("STMN06",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="208" priority="11" operator="containsText" text="STAN13">
+    <cfRule type="containsText" dxfId="396" priority="11" operator="containsText" text="STAN13">
       <formula>NOT(ISERROR(SEARCH("STAN13",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="207" priority="12" operator="containsText" text="STNN21">
+    <cfRule type="containsText" dxfId="395" priority="12" operator="containsText" text="STNN21">
       <formula>NOT(ISERROR(SEARCH("STNN21",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="206" priority="13" operator="containsText" text="LV">
+    <cfRule type="containsText" dxfId="394" priority="13" operator="containsText" text="LV">
       <formula>NOT(ISERROR(SEARCH("LV",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="205" priority="14" operator="containsText" text="TR">
+    <cfRule type="containsText" dxfId="393" priority="14" operator="containsText" text="TR">
       <formula>NOT(ISERROR(SEARCH("TR",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="204" priority="16" operator="containsText" text="NN13">
+    <cfRule type="containsText" dxfId="392" priority="16" operator="containsText" text="NN13">
       <formula>NOT(ISERROR(SEARCH("NN13",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="203" priority="20" operator="containsText" text="OFF">
+    <cfRule type="containsText" dxfId="391" priority="20" operator="containsText" text="OFF">
       <formula>NOT(ISERROR(SEARCH("OFF",F5)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -46214,117 +47826,117 @@
     <mergeCell ref="B22:C22"/>
   </mergeCells>
   <conditionalFormatting sqref="E5:AH10">
-    <cfRule type="containsText" dxfId="202" priority="23" operator="containsText" text="STN">
+    <cfRule type="containsText" dxfId="390" priority="23" operator="containsText" text="STN">
       <formula>NOT(ISERROR(SEARCH("STN",E5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="201" priority="24" operator="containsText" text="STN">
+    <cfRule type="containsText" dxfId="389" priority="24" operator="containsText" text="STN">
       <formula>NOT(ISERROR(SEARCH("STN",E5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="200" priority="25" operator="containsText" text="STM">
+    <cfRule type="containsText" dxfId="388" priority="25" operator="containsText" text="STM">
       <formula>NOT(ISERROR(SEARCH("STM",E5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="199" priority="26" operator="containsText" text="M">
+    <cfRule type="containsText" dxfId="387" priority="26" operator="containsText" text="M">
       <formula>NOT(ISERROR(SEARCH("M",E5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="198" priority="27" operator="containsText" text="STM1">
+    <cfRule type="containsText" dxfId="386" priority="27" operator="containsText" text="STM1">
       <formula>NOT(ISERROR(SEARCH("STM1",E5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="197" priority="28" operator="containsText" text="M">
+    <cfRule type="containsText" dxfId="385" priority="28" operator="containsText" text="M">
       <formula>NOT(ISERROR(SEARCH("M",E5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="196" priority="29" operator="containsText" text="STM">
+    <cfRule type="containsText" dxfId="384" priority="29" operator="containsText" text="STM">
       <formula>NOT(ISERROR(SEARCH("STM",E5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="195" priority="30" operator="containsText" text="STM">
+    <cfRule type="containsText" dxfId="383" priority="30" operator="containsText" text="STM">
       <formula>NOT(ISERROR(SEARCH("STM",E5)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E5:AH15">
-    <cfRule type="containsText" dxfId="194" priority="19" operator="containsText" text="A">
+    <cfRule type="containsText" dxfId="382" priority="19" operator="containsText" text="A">
       <formula>NOT(ISERROR(SEARCH("A",E5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="193" priority="5" operator="containsText" text="STM1">
+    <cfRule type="containsText" dxfId="381" priority="5" operator="containsText" text="STM1">
       <formula>NOT(ISERROR(SEARCH("STM1",E5)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E11:AH15">
-    <cfRule type="containsText" dxfId="192" priority="16" operator="containsText" text="STM1">
+    <cfRule type="containsText" dxfId="380" priority="16" operator="containsText" text="STM1">
       <formula>NOT(ISERROR(SEARCH("STM1",E11)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="191" priority="17" operator="containsText" text="O">
+    <cfRule type="containsText" dxfId="379" priority="17" operator="containsText" text="O">
       <formula>NOT(ISERROR(SEARCH("O",E11)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="190" priority="18" operator="containsText" text="N">
+    <cfRule type="containsText" dxfId="378" priority="18" operator="containsText" text="N">
       <formula>NOT(ISERROR(SEARCH("N",E11)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="189" priority="6" operator="containsText" text="STN">
+    <cfRule type="containsText" dxfId="377" priority="6" operator="containsText" text="STN">
       <formula>NOT(ISERROR(SEARCH("STN",E11)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="188" priority="7" operator="containsText" text="STN">
+    <cfRule type="containsText" dxfId="376" priority="7" operator="containsText" text="STN">
       <formula>NOT(ISERROR(SEARCH("STN",E11)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="187" priority="8" operator="containsText" text="STM">
+    <cfRule type="containsText" dxfId="375" priority="8" operator="containsText" text="STM">
       <formula>NOT(ISERROR(SEARCH("STM",E11)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="186" priority="9" operator="containsText" text="M">
+    <cfRule type="containsText" dxfId="374" priority="9" operator="containsText" text="M">
       <formula>NOT(ISERROR(SEARCH("M",E11)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="185" priority="10" operator="containsText" text="STM1">
+    <cfRule type="containsText" dxfId="373" priority="10" operator="containsText" text="STM1">
       <formula>NOT(ISERROR(SEARCH("STM1",E11)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="184" priority="11" operator="containsText" text="M">
+    <cfRule type="containsText" dxfId="372" priority="11" operator="containsText" text="M">
       <formula>NOT(ISERROR(SEARCH("M",E11)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="183" priority="12" operator="containsText" text="STM">
+    <cfRule type="containsText" dxfId="371" priority="12" operator="containsText" text="STM">
       <formula>NOT(ISERROR(SEARCH("STM",E11)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="182" priority="13" operator="containsText" text="STM">
+    <cfRule type="containsText" dxfId="370" priority="13" operator="containsText" text="STM">
       <formula>NOT(ISERROR(SEARCH("STM",E11)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="181" priority="14" operator="containsText" text="STM1">
+    <cfRule type="containsText" dxfId="369" priority="14" operator="containsText" text="STM1">
       <formula>NOT(ISERROR(SEARCH("STM1",E11)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="180" priority="15" operator="containsText" text="STA">
+    <cfRule type="containsText" dxfId="368" priority="15" operator="containsText" text="STA">
       <formula>NOT(ISERROR(SEARCH("STA",E11)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="179" priority="20" operator="containsText" text="M">
+    <cfRule type="containsText" dxfId="367" priority="20" operator="containsText" text="M">
       <formula>NOT(ISERROR(SEARCH("M",E11)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E5:AI15">
-    <cfRule type="containsText" dxfId="178" priority="3" operator="containsText" text="STM1">
+    <cfRule type="containsText" dxfId="366" priority="3" operator="containsText" text="STM1">
       <formula>NOT(ISERROR(SEARCH("STM1",E5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="177" priority="4" operator="containsText" text="STM1">
+    <cfRule type="containsText" dxfId="365" priority="4" operator="containsText" text="STM1">
       <formula>NOT(ISERROR(SEARCH("STM1",E5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="176" priority="1" operator="containsText" text="STN">
+    <cfRule type="containsText" dxfId="364" priority="1" operator="containsText" text="STN">
       <formula>NOT(ISERROR(SEARCH("STN",E5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="175" priority="2" operator="containsText" text="STA">
+    <cfRule type="containsText" dxfId="363" priority="2" operator="containsText" text="STA">
       <formula>NOT(ISERROR(SEARCH("STA",E5)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F5:AH5 E6:AH10">
-    <cfRule type="containsText" dxfId="174" priority="31" operator="containsText" text="STM1">
+    <cfRule type="containsText" dxfId="362" priority="31" operator="containsText" text="STM1">
       <formula>NOT(ISERROR(SEARCH("STM1",E5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="173" priority="32" operator="containsText" text="STA">
+    <cfRule type="containsText" dxfId="361" priority="32" operator="containsText" text="STA">
       <formula>NOT(ISERROR(SEARCH("STA",E5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="172" priority="33" operator="containsText" text="STM1">
+    <cfRule type="containsText" dxfId="360" priority="33" operator="containsText" text="STM1">
       <formula>NOT(ISERROR(SEARCH("STM1",E5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="171" priority="34" operator="containsText" text="O">
+    <cfRule type="containsText" dxfId="359" priority="34" operator="containsText" text="O">
       <formula>NOT(ISERROR(SEARCH("O",E5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="170" priority="35" operator="containsText" text="N">
+    <cfRule type="containsText" dxfId="358" priority="35" operator="containsText" text="N">
       <formula>NOT(ISERROR(SEARCH("N",E5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="169" priority="36" operator="containsText" text="A">
+    <cfRule type="containsText" dxfId="357" priority="36" operator="containsText" text="A">
       <formula>NOT(ISERROR(SEARCH("A",E5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="168" priority="37" operator="containsText" text="M">
+    <cfRule type="containsText" dxfId="356" priority="37" operator="containsText" text="M">
       <formula>NOT(ISERROR(SEARCH("M",E5)))</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>